<commit_message>
Restructure of Code Base
</commit_message>
<xml_diff>
--- a/backend/app/seed_data/users_import.xlsx
+++ b/backend/app/seed_data/users_import.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Users" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -727,7 +727,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>inv.manager</t>
+          <t>inventory.manager1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">

</xml_diff>